<commit_message>
Record Run 3: visit 1 with the lab machine's NVIDIA driver healed
Lab computer 03 runs NVIDIA's driver 535 with a prebuilt module. A desk
check of old-releases found that 23.04 cannot keep that combination: its
last prebuilt module needs driver 535.154.05, which 23.04 never got. If apt
had left the new kernel without a driver, the engine would still have said
healed, because its check reads only the release and dpkg's state.

So the EFI desktop VM got 03's NVIDIA packages at 03's versions, and visit
1 ran again. apt took the path that works: it installed the driver's dkms
package and built the module for both kernels, matching the driver. It
healed in 74 minutes, 26 more than without NVIDIA. The module loading on a
real card is left for 03.

Tested: Run 3 on KineticDesktop at 2415fcd
(evidence/ubuntu-22.10-2026-10-16-9.jsonl). Schema check passes; offline
292 + 48 + 19.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sf3000-tracker.xlsx
+++ b/docs/sf3000-tracker.xlsx
@@ -2218,22 +2218,22 @@
       <c r="L18" s="12" t="n"/>
       <c r="M18" s="12" t="inlineStr">
         <is>
-          <t>Ubuntu 22.10 (kinetic) → 23.04 (lunar) → 23.10 (mantic) → 24.04 (noble): visits 1 to 3; 24.04 → 26.04 (resolute) made to fail twice: Runs E and F; visit 4 restored after a held lock (2026-10-14); visit 4 healed at its second try (Run H, 2026-10-14) 22.10 → 23.04 on an EFI 22.10 desktop with stand-in Windows parts (KineticDesktop, 2026-10-16): healed, then failed on purpose and restored.</t>
+          <t>Ubuntu 22.10 (kinetic) → 23.04 (lunar) → 23.10 (mantic) → 24.04 (noble): visits 1 to 3; 24.04 → 26.04 (resolute) made to fail twice: Runs E and F; visit 4 restored after a held lock (2026-10-14); visit 4 healed at its second try (Run H, 2026-10-14) 22.10 → 23.04 on an EFI 22.10 desktop with stand-in Windows parts (KineticDesktop, 2026-10-16): healed, then failed on purpose and restored. With 03's NVIDIA 535 packages too (Run 3, 2026-10-16): healed; apt built the driver with dkms.</t>
         </is>
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
-          <t>Runs under the engine's procedure service: one y/N, then the upgrade, a reboot and the check. Since 2026-10-08: one upgrade per procedure and per visit (2-2.5 h lab slots, the person there); apt checked before the y/N; Timeshift installed by the engine if missing; /boot/efi left out of the snapshot (Windows' EFI partition on the lab's dual-boot machines); a step cut off by a power-off waits for the person (--run again offers the restore). Needs a snapshot: --take-snapshot (Timeshift; restored by itself if the upgrade fails, then checked) or --snapshot &lt;name&gt;. Precondition: apt works (eos-release-dead-repos healed). Written from the upgraders' source; plain do-release-upgrade would skip 23.04/23.10 and offer 24.04 directly from 22.10, which its upgrader is not built for. Timeshift 22.06.5 to 24.01.1 refuse '--tags O', so the engine passes no tags (2b09c29). Since 2026-10-09: dpkg's lock is held around the snapshot and the restore, and the snapshot is synced to disk (74340e2). Since 2026-10-10: /var/log/dist-upgrade is left out of the snapshot, so a failed upgrade's own logs survive the restore (main.log is the only place the non-interactive upgrader writes why it failed). Also since 2026-10-10: the engine keeps 256 MB set aside while a procedure runs and frees it first when a step fails, so a full disk cannot stop the restore (seen in Run F); and -26.04 is two steps, updates + reboot, then do-release-upgrade, which refuses while a kernel or libc6 update waits for a reboot. Run F found: the upgrader can exit while a dpkg it started still runs, and the engine, which then waited only for dpkg's frontend lock, started the restore with that dpkg running. Since 2026-10-11 (seen in Run G): before a restore the engine kills every other process in its service's cgroup (named in the record, leftovers_stopped), and it holds dpkg's own lock as well as the frontend's. Visit 4 (2026-10-14) found: the non-interactive upgrader says why it stopped only in its main.log, so a held dpkg lock read as a failed upgrade and was restored. Since then each upgrade step prints the end of that log when the upgrader fails, so the engine waits and retries instead (DESIGN §16; offline only). Run H (2026-10-14) found: the box before the y is worked out before the apt check, from apt's lists as they were, so on 24.04 it can say step 1 is done when new updates wait. Step 1 then runs anyway, since its own check finds them, and adds a reboot. Since 2026-10-14 the box is worked out again after the apt check, so it shows what the steps will find (DESIGN §16; offline only). On a desktop the upgrader runs in desktop mode whatever --mode=server says (main.log, 2026-10-16). Windows' parts unchanged by visit 1 and by its restore (check-windows.sh).</t>
+          <t>Runs under the engine's procedure service: one y/N, then the upgrade, a reboot and the check. Since 2026-10-08: one upgrade per procedure and per visit (2-2.5 h lab slots, the person there); apt checked before the y/N; Timeshift installed by the engine if missing; /boot/efi left out of the snapshot (Windows' EFI partition on the lab's dual-boot machines); a step cut off by a power-off waits for the person (--run again offers the restore). Needs a snapshot: --take-snapshot (Timeshift; restored by itself if the upgrade fails, then checked) or --snapshot &lt;name&gt;. Precondition: apt works (eos-release-dead-repos healed). Written from the upgraders' source; plain do-release-upgrade would skip 23.04/23.10 and offer 24.04 directly from 22.10, which its upgrader is not built for. Timeshift 22.06.5 to 24.01.1 refuse '--tags O', so the engine passes no tags (2b09c29). Since 2026-10-09: dpkg's lock is held around the snapshot and the restore, and the snapshot is synced to disk (74340e2). Since 2026-10-10: /var/log/dist-upgrade is left out of the snapshot, so a failed upgrade's own logs survive the restore (main.log is the only place the non-interactive upgrader writes why it failed). Also since 2026-10-10: the engine keeps 256 MB set aside while a procedure runs and frees it first when a step fails, so a full disk cannot stop the restore (seen in Run F); and -26.04 is two steps, updates + reboot, then do-release-upgrade, which refuses while a kernel or libc6 update waits for a reboot. Run F found: the upgrader can exit while a dpkg it started still runs, and the engine, which then waited only for dpkg's frontend lock, started the restore with that dpkg running. Since 2026-10-11 (seen in Run G): before a restore the engine kills every other process in its service's cgroup (named in the record, leftovers_stopped), and it holds dpkg's own lock as well as the frontend's. Visit 4 (2026-10-14) found: the non-interactive upgrader says why it stopped only in its main.log, so a held dpkg lock read as a failed upgrade and was restored. Since then each upgrade step prints the end of that log when the upgrader fails, so the engine waits and retries instead (DESIGN §16; offline only). Run H (2026-10-14) found: the box before the y is worked out before the apt check, from apt's lists as they were, so on 24.04 it can say step 1 is done when new updates wait. Step 1 then runs anyway, since its own check finds them, and adds a reboot. Since 2026-10-14 the box is worked out again after the apt check, so it shows what the steps will find (DESIGN §16; offline only). On a desktop the upgrader runs in desktop mode whatever --mode=server says (main.log, 2026-10-16). Windows' parts unchanged by visit 1 and by its restore (check-windows.sh). NVIDIA 535 on 23.04: the last prebuilt module needs 535.154.05, never released for 23.04, so the upgrade installs nvidia-dkms-535 535.146.02 and builds the module (needs kernel headers); 23.10 fits together again.</t>
         </is>
       </c>
       <c r="O18" s="12" t="inlineStr">
         <is>
-          <t>2026-10-16 · 22.10 → 23.04 on an EFI desktop · Run 1 healed in 48 min; Run 2 filled the disk mid-install and the engine restored 22.10 in about 1.5 min; nothing of Windows' changed either time</t>
+          <t>2026-10-16 · 22.10 → 23.04 on an EFI desktop · Run 1 healed in 48 min; Run 2 failed on purpose and was restored; Run 3, with 03's NVIDIA packages, healed in 74 min with the driver built by dkms; nothing of Windows' changed</t>
         </is>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
-          <t>Visit 1 on lab computer 03 (2026-10-21). Unseen on any VM: an NVIDIA driver through the upgrade; a lock that only the upgrader's log names.</t>
+          <t>Visit 1 on lab computer 03 (2026-10-21): check headers and Secure Boot first; after, nvidia-smi and dkms status. Unseen on any VM: the module loading on a real NVIDIA card; a lock that only the upgrader's log names.</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -6321,31 +6321,142 @@
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="10" t="n"/>
-      <c r="B73" s="10" t="n"/>
-      <c r="C73" s="10" t="n"/>
-      <c r="D73" s="10" t="n"/>
-      <c r="E73" s="10" t="n"/>
-      <c r="F73" s="10" t="n"/>
-      <c r="G73" s="10" t="n"/>
-    </row>
-    <row r="74" ht="210" customHeight="1">
-      <c r="A74" s="22" t="inlineStr">
-        <is>
-          <t>Times are IST (UTC+05:30). The logs themselves record UTC. Rows from 2026-09-07 23:35 to 2026-09-10 are records in evidence/ubuntu-26.04-2026-09-10.jsonl, copied off the VM on 2026-10-03; rows from 2026-10-04 are in evidence/ubuntu-26.04-2026-10-04.jsonl, rows from 2026-10-06 in evidence/ubuntu-26.04-2026-10-06.jsonl, and rows from 2026-10-07 in evidence/ubuntu-22.10-2026-10-07.jsonl and, from 12:13, evidence/ubuntu-22.10-2026-10-07-2.jsonl (the 22.10 VM, KineticServer). Rows from 2026-10-08 19:56 are the procedure runs, in evidence/ubuntu-22.10-2026-10-09.jsonl, copied from the service's own log, /var/log/sf3000/runs.jsonl. Rows from 2026-10-10 15:15 and 15:16 are lines 10 to 12 of evidence/ubuntu-22.10-2026-10-10.jsonl, whose first nine lines are the 2026-10-09 file again. Rows from 2026-10-10 16:33 are visit 1 of the upgrade, in evidence/ubuntu-22.10-2026-10-10-2.jsonl. The row from 18:40 is visit 2, line 3 of evidence/ubuntu-22.10-2026-10-10-3.jsonl, whose first two lines are visit 1's file again. The row from 20:00 is visit 3, line 4 of evidence/ubuntu-22.10-2026-10-10-4.jsonl, whose first three lines are visit 2's file again. The rows from 23:26 and 23:42 are Runs E and F, lines 5 and 6 of evidence/ubuntu-22.10-2026-10-10-5.jsonl, whose first four lines are visit 3's file again. The row from 2026-10-11 01:13 is Run G, line 7 of evidence/ubuntu-22.10-2026-10-11.jsonl, whose first six lines are the 2026-10-10 -5 file again. The rows from 2026-10-14 17:09 and 17:13 are visit 4, lines 8 and 9 of evidence/ubuntu-22.10-2026-10-14.jsonl, whose first seven lines are the 2026-10-11 file again. The rows from 2026-10-14 19:09 and 19:12 are Run H, lines 10 and 11 of evidence/ubuntu-22.10-2026-10-14-2.jsonl, whose first nine lines are the 2026-10-14 file again. Rows whose Evidence says 'Terminal output' have no record: the engine refuses before it logs anything, or the row is a sweep, which never logs. The six rows before 2026-09-07 23:35 come from commit messages: the VM's log was reset on the evening of 2026-09-07, before anyone copied it. Add one row per run from now on, pointing at its evidence file and line. The rows from 2026-10-16 17:10 to 17:17 are Run 1 of tests/efi-proof on KineticDesktop, an EFI 22.10 desktop VM, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16.jsonl. The rows from 18:03 to 18:10 are Run 2, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-2.jsonl: a file of its own, because the VM went back to its efi-ready snapshot between the runs. The rows from 2026-10-16 19:29 to 19:46 are tests/grub-windows-proof on KineticDesktop, one record each in evidence/ubuntu-22.10-2026-10-16-3.jsonl to -8.jsonl: each run began from a snapshot restore, which deletes the clone's run log.</t>
-        </is>
-      </c>
-      <c r="B74" s="23" t="n"/>
-      <c r="C74" s="23" t="n"/>
-      <c r="D74" s="23" t="n"/>
-      <c r="E74" s="23" t="n"/>
-      <c r="F74" s="23" t="n"/>
-      <c r="G74" s="24" t="n"/>
+    <row r="73" ht="56" customHeight="1">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 20:02</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>2415fcd</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>engine/install</t>
+        </is>
+      </c>
+      <c r="E73" s="10" t="inlineStr">
+        <is>
+          <t>installed</t>
+        </is>
+      </c>
+      <c r="F73" s="10" t="inlineStr">
+        <is>
+          <t>Run 3 of tests/efi-proof, on KineticDesktop from VBox snapshot efi-nvidia: efi-ready plus lab computer 03's NVIDIA packages at 03's versions (nvidia-driver-535 535.54.03, prebuilt linux-modules-nvidia-535-generic-hwe-22.04 5.19.0-46, no dkms). python3-jsonschema installed after a y.</t>
+        </is>
+      </c>
+      <c r="G73" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-16-9.jsonl, line 1; install.log, copied off</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="56" customHeight="1">
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 20:03</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>2415fcd</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>release-upgrade-to-23.04/install</t>
+        </is>
+      </c>
+      <c r="E74" s="10" t="inlineStr">
+        <is>
+          <t>installed</t>
+        </is>
+      </c>
+      <c r="F74" s="10" t="inlineStr">
+        <is>
+          <t>Run 3: Timeshift installed after the y at the box.</t>
+        </is>
+      </c>
+      <c r="G74" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-16-9.jsonl, line 2; install.log, copied off</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="56" customHeight="1">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 20:08</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>22.10 → 23.04</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>2415fcd</t>
+        </is>
+      </c>
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>release-upgrade-to-23.04/to-23.04</t>
+        </is>
+      </c>
+      <c r="E75" s="10" t="inlineStr">
+        <is>
+          <t>healed</t>
+        </is>
+      </c>
+      <c r="F75" s="10" t="inlineStr">
+        <is>
+          <t>Run 3: visit 1 with 03's NVIDIA packages. Snapshot 2026-10-16_20-03-04 (6 min, of 22.10 packages:758d752e41e5d906). 23.04's last prebuilt module needs driver 535.154.05, which 23.04 never got, so apt installed nvidia-dkms-535 535.146.02 with dkms and a compiler; dkms built the module for 6.2.0-39 and 5.19.0-46, matching the driver. Main install pass 34 min (17 in Run 1). Check after: 2304; 74 min from the y. GNOME's login screen; the VM has no NVIDIA card. check-windows.sh: the same two Ubuntu changes as Run 1, nothing else.</t>
+        </is>
+      </c>
+      <c r="G75" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-16-9.jsonl, line 3; the upgrader's logs, dkms status and the check-windows files (logs/kinetic-desktop-run-3), copied off</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="n"/>
+      <c r="B76" s="10" t="n"/>
+      <c r="C76" s="10" t="n"/>
+      <c r="D76" s="10" t="n"/>
+      <c r="E76" s="10" t="n"/>
+      <c r="F76" s="10" t="n"/>
+      <c r="G76" s="10" t="n"/>
+    </row>
+    <row r="77" ht="225" customHeight="1">
+      <c r="A77" s="22" t="inlineStr">
+        <is>
+          <t>Times are IST (UTC+05:30). The logs themselves record UTC. Rows from 2026-09-07 23:35 to 2026-09-10 are records in evidence/ubuntu-26.04-2026-09-10.jsonl, copied off the VM on 2026-10-03; rows from 2026-10-04 are in evidence/ubuntu-26.04-2026-10-04.jsonl, rows from 2026-10-06 in evidence/ubuntu-26.04-2026-10-06.jsonl, and rows from 2026-10-07 in evidence/ubuntu-22.10-2026-10-07.jsonl and, from 12:13, evidence/ubuntu-22.10-2026-10-07-2.jsonl (the 22.10 VM, KineticServer). Rows from 2026-10-08 19:56 are the procedure runs, in evidence/ubuntu-22.10-2026-10-09.jsonl, copied from the service's own log, /var/log/sf3000/runs.jsonl. Rows from 2026-10-10 15:15 and 15:16 are lines 10 to 12 of evidence/ubuntu-22.10-2026-10-10.jsonl, whose first nine lines are the 2026-10-09 file again. Rows from 2026-10-10 16:33 are visit 1 of the upgrade, in evidence/ubuntu-22.10-2026-10-10-2.jsonl. The row from 18:40 is visit 2, line 3 of evidence/ubuntu-22.10-2026-10-10-3.jsonl, whose first two lines are visit 1's file again. The row from 20:00 is visit 3, line 4 of evidence/ubuntu-22.10-2026-10-10-4.jsonl, whose first three lines are visit 2's file again. The rows from 23:26 and 23:42 are Runs E and F, lines 5 and 6 of evidence/ubuntu-22.10-2026-10-10-5.jsonl, whose first four lines are visit 3's file again. The row from 2026-10-11 01:13 is Run G, line 7 of evidence/ubuntu-22.10-2026-10-11.jsonl, whose first six lines are the 2026-10-10 -5 file again. The rows from 2026-10-14 17:09 and 17:13 are visit 4, lines 8 and 9 of evidence/ubuntu-22.10-2026-10-14.jsonl, whose first seven lines are the 2026-10-11 file again. The rows from 2026-10-14 19:09 and 19:12 are Run H, lines 10 and 11 of evidence/ubuntu-22.10-2026-10-14-2.jsonl, whose first nine lines are the 2026-10-14 file again. Rows whose Evidence says 'Terminal output' have no record: the engine refuses before it logs anything, or the row is a sweep, which never logs. The six rows before 2026-09-07 23:35 come from commit messages: the VM's log was reset on the evening of 2026-09-07, before anyone copied it. Add one row per run from now on, pointing at its evidence file and line. The rows from 2026-10-16 17:10 to 17:17 are Run 1 of tests/efi-proof on KineticDesktop, an EFI 22.10 desktop VM, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16.jsonl. The rows from 18:03 to 18:10 are Run 2, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-2.jsonl: a file of its own, because the VM went back to its efi-ready snapshot between the runs. The rows from 2026-10-16 19:29 to 19:46 are tests/grub-windows-proof on KineticDesktop, one record each in evidence/ubuntu-22.10-2026-10-16-3.jsonl to -8.jsonl: each run began from a snapshot restore, which deletes the clone's run log. The rows from 2026-10-16 20:02 to 20:08 are Run 3 of tests/efi-proof, with 03's NVIDIA packages, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-9.jsonl.</t>
+        </is>
+      </c>
+      <c r="B77" s="23" t="n"/>
+      <c r="C77" s="23" t="n"/>
+      <c r="D77" s="23" t="n"/>
+      <c r="E77" s="23" t="n"/>
+      <c r="F77" s="23" t="n"/>
+      <c r="G77" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A74:G74"/>
+    <mergeCell ref="A77:G77"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record --cancel after a real cut-off, the first on a VM
Lab computer 03's run of 2026-10-14 was cut off, so on visit day its first
step is --cancel. That had never run after a real cut-off. On the EFI
desktop VM, a test step was cut off by a power-off; the boot after held it
for a person, and --cancel recorded interrupted, kept the Timeshift snapshot
and restored nothing. The lab kit's new before-visit check said STOP while
the cut-off was held, and READY after.

Tested: on KineticDesktop at d4a34a0, with the lab kit's scripts
(evidence/ubuntu-22.10-2026-10-16-10.jsonl). Schema check passes. The
engine is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sf3000-tracker.xlsx
+++ b/docs/sf3000-tracker.xlsx
@@ -3661,7 +3661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -6432,31 +6432,142 @@
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="10" t="n"/>
-      <c r="B76" s="10" t="n"/>
-      <c r="C76" s="10" t="n"/>
-      <c r="D76" s="10" t="n"/>
-      <c r="E76" s="10" t="n"/>
-      <c r="F76" s="10" t="n"/>
-      <c r="G76" s="10" t="n"/>
-    </row>
-    <row r="77" ht="225" customHeight="1">
-      <c r="A77" s="22" t="inlineStr">
-        <is>
-          <t>Times are IST (UTC+05:30). The logs themselves record UTC. Rows from 2026-09-07 23:35 to 2026-09-10 are records in evidence/ubuntu-26.04-2026-09-10.jsonl, copied off the VM on 2026-10-03; rows from 2026-10-04 are in evidence/ubuntu-26.04-2026-10-04.jsonl, rows from 2026-10-06 in evidence/ubuntu-26.04-2026-10-06.jsonl, and rows from 2026-10-07 in evidence/ubuntu-22.10-2026-10-07.jsonl and, from 12:13, evidence/ubuntu-22.10-2026-10-07-2.jsonl (the 22.10 VM, KineticServer). Rows from 2026-10-08 19:56 are the procedure runs, in evidence/ubuntu-22.10-2026-10-09.jsonl, copied from the service's own log, /var/log/sf3000/runs.jsonl. Rows from 2026-10-10 15:15 and 15:16 are lines 10 to 12 of evidence/ubuntu-22.10-2026-10-10.jsonl, whose first nine lines are the 2026-10-09 file again. Rows from 2026-10-10 16:33 are visit 1 of the upgrade, in evidence/ubuntu-22.10-2026-10-10-2.jsonl. The row from 18:40 is visit 2, line 3 of evidence/ubuntu-22.10-2026-10-10-3.jsonl, whose first two lines are visit 1's file again. The row from 20:00 is visit 3, line 4 of evidence/ubuntu-22.10-2026-10-10-4.jsonl, whose first three lines are visit 2's file again. The rows from 23:26 and 23:42 are Runs E and F, lines 5 and 6 of evidence/ubuntu-22.10-2026-10-10-5.jsonl, whose first four lines are visit 3's file again. The row from 2026-10-11 01:13 is Run G, line 7 of evidence/ubuntu-22.10-2026-10-11.jsonl, whose first six lines are the 2026-10-10 -5 file again. The rows from 2026-10-14 17:09 and 17:13 are visit 4, lines 8 and 9 of evidence/ubuntu-22.10-2026-10-14.jsonl, whose first seven lines are the 2026-10-11 file again. The rows from 2026-10-14 19:09 and 19:12 are Run H, lines 10 and 11 of evidence/ubuntu-22.10-2026-10-14-2.jsonl, whose first nine lines are the 2026-10-14 file again. Rows whose Evidence says 'Terminal output' have no record: the engine refuses before it logs anything, or the row is a sweep, which never logs. The six rows before 2026-09-07 23:35 come from commit messages: the VM's log was reset on the evening of 2026-09-07, before anyone copied it. Add one row per run from now on, pointing at its evidence file and line. The rows from 2026-10-16 17:10 to 17:17 are Run 1 of tests/efi-proof on KineticDesktop, an EFI 22.10 desktop VM, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16.jsonl. The rows from 18:03 to 18:10 are Run 2, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-2.jsonl: a file of its own, because the VM went back to its efi-ready snapshot between the runs. The rows from 2026-10-16 19:29 to 19:46 are tests/grub-windows-proof on KineticDesktop, one record each in evidence/ubuntu-22.10-2026-10-16-3.jsonl to -8.jsonl: each run began from a snapshot restore, which deletes the clone's run log. The rows from 2026-10-16 20:02 to 20:08 are Run 3 of tests/efi-proof, with 03's NVIDIA packages, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-9.jsonl.</t>
-        </is>
-      </c>
-      <c r="B77" s="23" t="n"/>
-      <c r="C77" s="23" t="n"/>
-      <c r="D77" s="23" t="n"/>
-      <c r="E77" s="23" t="n"/>
-      <c r="F77" s="23" t="n"/>
-      <c r="G77" s="24" t="n"/>
+    <row r="76" ht="56" customHeight="1">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 22:07</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>d4a34a0</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>engine/install</t>
+        </is>
+      </c>
+      <c r="E76" s="10" t="inlineStr">
+        <is>
+          <t>installed</t>
+        </is>
+      </c>
+      <c r="F76" s="10" t="inlineStr">
+        <is>
+          <t>The lab kit's new scripts on KineticDesktop from efi-nvidia, in visit day's order: 2-get-engine (pulled to d4a34a0), 6-before-visit (STOP: no jsonschema), then 3-sweep installed python3-jsonschema after a y.</t>
+        </is>
+      </c>
+      <c r="G76" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-16-10.jsonl, line 1; the kit's out folder, copied off</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="56" customHeight="1">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 22:10</t>
+        </is>
+      </c>
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>d4a34a0</t>
+        </is>
+      </c>
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>cut-off-proof/install</t>
+        </is>
+      </c>
+      <c r="E77" s="10" t="inlineStr">
+        <is>
+          <t>installed</t>
+        </is>
+      </c>
+      <c r="F77" s="10" t="inlineStr">
+        <is>
+          <t>Before the real cut-off: Timeshift installed for cut-off-proof --take-snapshot.</t>
+        </is>
+      </c>
+      <c r="G77" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-16-10.jsonl, line 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="56" customHeight="1">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 22:15</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>d4a34a0</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>cut-off-proof/long</t>
+        </is>
+      </c>
+      <c r="E78" s="10" t="inlineStr">
+        <is>
+          <t>interrupted</t>
+        </is>
+      </c>
+      <c r="F78" s="10" t="inlineStr">
+        <is>
+          <t>--cancel after a real cut-off, the first on a VM: the VM powered off a minute into step long; the boot after held it (cut_off) and the kit's 6-before-visit said STOP. sudo python3 engine/runner.py --cancel asked nothing and recorded 'not attempted: cancelled by hand; Timeshift snapshot 2026-10-16_22-10-13 kept'. Nothing restored; the snapshot kept. Then 6 said READY. Lab computer 03's first step on 2026-10-21. (The timestamp is the step's start.)</t>
+        </is>
+      </c>
+      <c r="G78" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-16-10.jsonl, line 3; journal and kit output (logs/kinetic-desktop-cancel), copied off</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="n"/>
+      <c r="B79" s="10" t="n"/>
+      <c r="C79" s="10" t="n"/>
+      <c r="D79" s="10" t="n"/>
+      <c r="E79" s="10" t="n"/>
+      <c r="F79" s="10" t="n"/>
+      <c r="G79" s="10" t="n"/>
+    </row>
+    <row r="80" ht="240" customHeight="1">
+      <c r="A80" s="22" t="inlineStr">
+        <is>
+          <t>Times are IST (UTC+05:30). The logs themselves record UTC. Rows from 2026-09-07 23:35 to 2026-09-10 are records in evidence/ubuntu-26.04-2026-09-10.jsonl, copied off the VM on 2026-10-03; rows from 2026-10-04 are in evidence/ubuntu-26.04-2026-10-04.jsonl, rows from 2026-10-06 in evidence/ubuntu-26.04-2026-10-06.jsonl, and rows from 2026-10-07 in evidence/ubuntu-22.10-2026-10-07.jsonl and, from 12:13, evidence/ubuntu-22.10-2026-10-07-2.jsonl (the 22.10 VM, KineticServer). Rows from 2026-10-08 19:56 are the procedure runs, in evidence/ubuntu-22.10-2026-10-09.jsonl, copied from the service's own log, /var/log/sf3000/runs.jsonl. Rows from 2026-10-10 15:15 and 15:16 are lines 10 to 12 of evidence/ubuntu-22.10-2026-10-10.jsonl, whose first nine lines are the 2026-10-09 file again. Rows from 2026-10-10 16:33 are visit 1 of the upgrade, in evidence/ubuntu-22.10-2026-10-10-2.jsonl. The row from 18:40 is visit 2, line 3 of evidence/ubuntu-22.10-2026-10-10-3.jsonl, whose first two lines are visit 1's file again. The row from 20:00 is visit 3, line 4 of evidence/ubuntu-22.10-2026-10-10-4.jsonl, whose first three lines are visit 2's file again. The rows from 23:26 and 23:42 are Runs E and F, lines 5 and 6 of evidence/ubuntu-22.10-2026-10-10-5.jsonl, whose first four lines are visit 3's file again. The row from 2026-10-11 01:13 is Run G, line 7 of evidence/ubuntu-22.10-2026-10-11.jsonl, whose first six lines are the 2026-10-10 -5 file again. The rows from 2026-10-14 17:09 and 17:13 are visit 4, lines 8 and 9 of evidence/ubuntu-22.10-2026-10-14.jsonl, whose first seven lines are the 2026-10-11 file again. The rows from 2026-10-14 19:09 and 19:12 are Run H, lines 10 and 11 of evidence/ubuntu-22.10-2026-10-14-2.jsonl, whose first nine lines are the 2026-10-14 file again. Rows whose Evidence says 'Terminal output' have no record: the engine refuses before it logs anything, or the row is a sweep, which never logs. The six rows before 2026-09-07 23:35 come from commit messages: the VM's log was reset on the evening of 2026-09-07, before anyone copied it. Add one row per run from now on, pointing at its evidence file and line. The rows from 2026-10-16 17:10 to 17:17 are Run 1 of tests/efi-proof on KineticDesktop, an EFI 22.10 desktop VM, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16.jsonl. The rows from 18:03 to 18:10 are Run 2, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-2.jsonl: a file of its own, because the VM went back to its efi-ready snapshot between the runs. The rows from 2026-10-16 19:29 to 19:46 are tests/grub-windows-proof on KineticDesktop, one record each in evidence/ubuntu-22.10-2026-10-16-3.jsonl to -8.jsonl: each run began from a snapshot restore, which deletes the clone's run log. The rows from 2026-10-16 20:02 to 20:08 are Run 3 of tests/efi-proof, with 03's NVIDIA packages, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-9.jsonl. The rows from 2026-10-16 22:07 to 22:15 are the lab kit's test and --cancel after a real cut-off, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-10.jsonl.</t>
+        </is>
+      </c>
+      <c r="B80" s="23" t="n"/>
+      <c r="C80" s="23" t="n"/>
+      <c r="D80" s="23" t="n"/>
+      <c r="E80" s="23" t="n"/>
+      <c r="F80" s="23" t="n"/>
+      <c r="G80" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A77:G77"/>
+    <mergeCell ref="A80:G80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Run the box with a summary on the EFI desktop VM
The box with a summary had been checked offline only. On KineticDesktop,
from grub-trap, it did what the offline checks said. The sweep and the box
showed windows-missing-from-grub's summary and no command; the box was
14 lines. v printed the command and the source, and n then changed
nothing (declined). y healed in 4.9 s, and the engine printed "running
the fix", not the command. Both records hold the full command. Windows'
parts matched the record from before the trap.

Also seen: after a warm reboot, GRUB's 10 s countdown passed in about
3 s on this host, so the demo notes now say to press an arrow key to hold
the menu.

Tested: on KineticDesktop at a298fc9 (evidence/ubuntu-22.10-2026-10-25.jsonl).
Schema check passes. The engine is unchanged since a298fc9.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sf3000-tracker.xlsx
+++ b/docs/sf3000-tracker.xlsx
@@ -2290,7 +2290,7 @@
       </c>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>Proven on the EFI 22.10 desktop VM (2026-10-16): healed 3 times (twice at aff2c9c, once at 279952d, about 5 s each)</t>
+          <t>Proven on the EFI 22.10 desktop VM (2026-10-16): healed 3 times (twice at aff2c9c, once at 279952d, about 5 s each); healed again on 2026-10-25 at a298fc9 (4.9 s), with its summary in the box</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="N19" s="12" t="inlineStr">
         <is>
-          <t>Ubuntu's 'auto' hides Windows for good after one rebuild without it. A stale Windows entry reads PROBLEM; the verify then undoes the fix. grub.cfg at 0600 (GRUB password): ERROR for a user. A cold start straight after a VBox restore skipped the menu on this host: demo with a warm reboot.</t>
+          <t>Ubuntu's 'auto' hides Windows for good after one rebuild without it. A stale Windows entry reads PROBLEM; the verify then undoes the fix. grub.cfg at 0600 (GRUB password): ERROR for a user. A cold start straight after a VBox restore skipped the menu on this host: demo with a warm reboot. On 2026-10-25 a warm reboot showed the menu for only about 3 s (the countdown ran fast): press an arrow key to hold it.</t>
         </is>
       </c>
       <c r="O19" s="12" t="inlineStr">
         <is>
-          <t>2026-10-16 · 22.10 · healed in 5.1 s; undone when it could not work and when it stopped early (Runs 4-6, 279952d)</t>
+          <t>2026-10-25 · 22.10 · the box with a summary: v then n declined; y healed in 4.9 s (a298fc9)</t>
         </is>
       </c>
       <c r="P19" s="12" t="inlineStr">
@@ -3661,7 +3661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -6728,23 +6728,97 @@
         </is>
       </c>
     </row>
-    <row r="84"/>
-    <row r="85" ht="270" customHeight="1">
-      <c r="A85" s="22" t="inlineStr">
-        <is>
-          <t>Times are IST (UTC+05:30). The logs themselves record UTC. Rows from 2026-09-07 23:35 to 2026-09-10 are records in evidence/ubuntu-26.04-2026-09-10.jsonl, copied off the VM on 2026-10-03; rows from 2026-10-04 are in evidence/ubuntu-26.04-2026-10-04.jsonl, rows from 2026-10-06 in evidence/ubuntu-26.04-2026-10-06.jsonl, and rows from 2026-10-07 in evidence/ubuntu-22.10-2026-10-07.jsonl and, from 12:13, evidence/ubuntu-22.10-2026-10-07-2.jsonl (the 22.10 VM, KineticServer). Rows from 2026-10-08 19:56 are the procedure runs, in evidence/ubuntu-22.10-2026-10-09.jsonl, copied from the service's own log, /var/log/sf3000/runs.jsonl. Rows from 2026-10-10 15:15 and 15:16 are lines 10 to 12 of evidence/ubuntu-22.10-2026-10-10.jsonl, whose first nine lines are the 2026-10-09 file again. Rows from 2026-10-10 16:33 are visit 1 of the upgrade, in evidence/ubuntu-22.10-2026-10-10-2.jsonl. The row from 18:40 is visit 2, line 3 of evidence/ubuntu-22.10-2026-10-10-3.jsonl, whose first two lines are visit 1's file again. The row from 20:00 is visit 3, line 4 of evidence/ubuntu-22.10-2026-10-10-4.jsonl, whose first three lines are visit 2's file again. The rows from 23:26 and 23:42 are Runs E and F, lines 5 and 6 of evidence/ubuntu-22.10-2026-10-10-5.jsonl, whose first four lines are visit 3's file again. The row from 2026-10-11 01:13 is Run G, line 7 of evidence/ubuntu-22.10-2026-10-11.jsonl, whose first six lines are the 2026-10-10 -5 file again. The rows from 2026-10-14 17:09 and 17:13 are visit 4, lines 8 and 9 of evidence/ubuntu-22.10-2026-10-14.jsonl, whose first seven lines are the 2026-10-11 file again. The rows from 2026-10-14 19:09 and 19:12 are Run H, lines 10 and 11 of evidence/ubuntu-22.10-2026-10-14-2.jsonl, whose first nine lines are the 2026-10-14 file again. Rows whose Evidence says 'Terminal output' have no record: the engine refuses before it logs anything, or the row is a sweep, which never logs. The six rows before 2026-09-07 23:35 come from commit messages: the VM's log was reset on the evening of 2026-09-07, before anyone copied it. Add one row per run from now on, pointing at its evidence file and line. The rows from 2026-10-16 17:10 to 17:17 are Run 1 of tests/efi-proof on KineticDesktop, an EFI 22.10 desktop VM, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16.jsonl. The rows from 18:03 to 18:10 are Run 2, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-2.jsonl: a file of its own, because the VM went back to its efi-ready snapshot between the runs. The rows from 2026-10-16 19:29 to 19:46 are tests/grub-windows-proof on KineticDesktop, one record each in evidence/ubuntu-22.10-2026-10-16-3.jsonl to -8.jsonl: each run began from a snapshot restore, which deletes the clone's run log. The rows from 2026-10-16 20:02 to 20:08 are Run 3 of tests/efi-proof, with 03's NVIDIA packages, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-9.jsonl. The rows from 2026-10-16 22:07 to 22:15 are the lab kit's test and --cancel after a real cut-off, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-10.jsonl. The rows from 2026-10-14 14:07 to 2026-10-21 13:52 are lab computer MITB-IT-406-03, a real lab machine: lines 1 to 4 of evidence/lab-MITB-IT-406-03-ubuntu-22.10-2026-10-21.jsonl (its /var/log/sf3000/runs.jsonl) and line 1 of evidence/lab-MITB-IT-406-03-ubuntu-22.10-2026-10-14.jsonl (its clone's logs/runs.jsonl). Its clock is 5 h 28 min fast; their times are corrected to the real time.</t>
-        </is>
-      </c>
-      <c r="B85" s="23" t="n"/>
-      <c r="C85" s="23" t="n"/>
-      <c r="D85" s="23" t="n"/>
-      <c r="E85" s="23" t="n"/>
-      <c r="F85" s="23" t="n"/>
-      <c r="G85" s="24" t="n"/>
+    <row r="84" ht="70" customHeight="1">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-25 14:59</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>a298fc9</t>
+        </is>
+      </c>
+      <c r="D84" s="10" t="inlineStr">
+        <is>
+          <t>windows-missing-from-grub</t>
+        </is>
+      </c>
+      <c r="E84" s="10" t="inlineStr">
+        <is>
+          <t>declined</t>
+        </is>
+      </c>
+      <c r="F84" s="10" t="inlineStr">
+        <is>
+          <t>Run 7 (tests/grub-windows-proof), on KineticDesktop from grub-trap: the box with a summary. The sweep and the box showed the summary, not the command; the box was 14 lines. v printed the command and the source, then asked again; answered n. /etc/default/grub unchanged (e7e2c4ab...), no backup made.</t>
+        </is>
+      </c>
+      <c r="G84" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-25.jsonl, line 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="70" customHeight="1">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-25 14:59</t>
+        </is>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>a298fc9</t>
+        </is>
+      </c>
+      <c r="D85" s="10" t="inlineStr">
+        <is>
+          <t>windows-missing-from-grub</t>
+        </is>
+      </c>
+      <c r="E85" s="10" t="inlineStr">
+        <is>
+          <t>healed</t>
+        </is>
+      </c>
+      <c r="F85" s="10" t="inlineStr">
+        <is>
+          <t>Run 8: answered y at the box. The engine printed 'running the fix', not the command. 1 → 0 in 4.9 s. check-windows after the fix matched the record from before the trap. A warm reboot showed the menu with Windows, but its 10 s countdown passed in about 3 s (the host's virtual clock).</t>
+        </is>
+      </c>
+      <c r="G85" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-25.jsonl, line 2; console, screenshots and Windows checks in logs/confirm-summary-run-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86"/>
+    <row r="87" ht="270" customHeight="1">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>Times are IST (UTC+05:30). The logs themselves record UTC. Rows from 2026-09-07 23:35 to 2026-09-10 are records in evidence/ubuntu-26.04-2026-09-10.jsonl, copied off the VM on 2026-10-03; rows from 2026-10-04 are in evidence/ubuntu-26.04-2026-10-04.jsonl, rows from 2026-10-06 in evidence/ubuntu-26.04-2026-10-06.jsonl, and rows from 2026-10-07 in evidence/ubuntu-22.10-2026-10-07.jsonl and, from 12:13, evidence/ubuntu-22.10-2026-10-07-2.jsonl (the 22.10 VM, KineticServer). Rows from 2026-10-08 19:56 are the procedure runs, in evidence/ubuntu-22.10-2026-10-09.jsonl, copied from the service's own log, /var/log/sf3000/runs.jsonl. Rows from 2026-10-10 15:15 and 15:16 are lines 10 to 12 of evidence/ubuntu-22.10-2026-10-10.jsonl, whose first nine lines are the 2026-10-09 file again. Rows from 2026-10-10 16:33 are visit 1 of the upgrade, in evidence/ubuntu-22.10-2026-10-10-2.jsonl. The row from 18:40 is visit 2, line 3 of evidence/ubuntu-22.10-2026-10-10-3.jsonl, whose first two lines are visit 1's file again. The row from 20:00 is visit 3, line 4 of evidence/ubuntu-22.10-2026-10-10-4.jsonl, whose first three lines are visit 2's file again. The rows from 23:26 and 23:42 are Runs E and F, lines 5 and 6 of evidence/ubuntu-22.10-2026-10-10-5.jsonl, whose first four lines are visit 3's file again. The row from 2026-10-11 01:13 is Run G, line 7 of evidence/ubuntu-22.10-2026-10-11.jsonl, whose first six lines are the 2026-10-10 -5 file again. The rows from 2026-10-14 17:09 and 17:13 are visit 4, lines 8 and 9 of evidence/ubuntu-22.10-2026-10-14.jsonl, whose first seven lines are the 2026-10-11 file again. The rows from 2026-10-14 19:09 and 19:12 are Run H, lines 10 and 11 of evidence/ubuntu-22.10-2026-10-14-2.jsonl, whose first nine lines are the 2026-10-14 file again. Rows whose Evidence says 'Terminal output' have no record: the engine refuses before it logs anything, or the row is a sweep, which never logs. The six rows before 2026-09-07 23:35 come from commit messages: the VM's log was reset on the evening of 2026-09-07, before anyone copied it. Add one row per run from now on, pointing at its evidence file and line. The rows from 2026-10-16 17:10 to 17:17 are Run 1 of tests/efi-proof on KineticDesktop, an EFI 22.10 desktop VM, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16.jsonl. The rows from 18:03 to 18:10 are Run 2, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-2.jsonl: a file of its own, because the VM went back to its efi-ready snapshot between the runs. The rows from 2026-10-16 19:29 to 19:46 are tests/grub-windows-proof on KineticDesktop, one record each in evidence/ubuntu-22.10-2026-10-16-3.jsonl to -8.jsonl: each run began from a snapshot restore, which deletes the clone's run log. The rows from 2026-10-16 20:02 to 20:08 are Run 3 of tests/efi-proof, with 03's NVIDIA packages, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-9.jsonl. The rows from 2026-10-16 22:07 to 22:15 are the lab kit's test and --cancel after a real cut-off, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-10.jsonl. The rows from 2026-10-14 14:07 to 2026-10-21 13:52 are lab computer MITB-IT-406-03, a real lab machine: lines 1 to 4 of evidence/lab-MITB-IT-406-03-ubuntu-22.10-2026-10-21.jsonl (its /var/log/sf3000/runs.jsonl) and line 1 of evidence/lab-MITB-IT-406-03-ubuntu-22.10-2026-10-14.jsonl (its clone's logs/runs.jsonl). Its clock is 5 h 28 min fast; their times are corrected to the real time. The rows from 2026-10-25 14:59 are Runs 7 and 8 of tests/grub-windows-proof, the box with a summary (branch confirm-summary, a298fc9), lines 1 and 2 of evidence/ubuntu-22.10-2026-10-25.jsonl.</t>
+        </is>
+      </c>
+      <c r="B87" s="23" t="n"/>
+      <c r="C87" s="23" t="n"/>
+      <c r="D87" s="23" t="n"/>
+      <c r="E87" s="23" t="n"/>
+      <c r="F87" s="23" t="n"/>
+      <c r="G87" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A85:G85"/>
+    <mergeCell ref="A87:G87"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rehearse the live demo on the EFI desktop VM, and time it
The demo on 2026-11-03 will be all live, with no pre-recorded clip. A
timed rehearsal from a new VBox snapshot, demo-start (grub-trap with the
clone at c4d67cc), checks that it fits. Machine time was about 2 min 40 s:
the reboot with the fault 50 s, sweep 3 s, fix 14 s, the reboot after 44 s,
check-windows 47 s. The fix healed, and Windows' parts were unchanged.

GRUB's menu is up for only about 0.6 s on this host, not 3 s as first
thought. Tapping Up from the VirtualBox logo on stops the countdown before
the menu draws, and the menu then stays until Enter. The demo notes say so.

Tested: on KineticDesktop at c4d67cc (evidence/ubuntu-22.10-2026-10-25-2.jsonl).
Schema check passes. The engine is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sf3000-tracker.xlsx
+++ b/docs/sf3000-tracker.xlsx
@@ -2305,7 +2305,7 @@
       </c>
       <c r="N19" s="12" t="inlineStr">
         <is>
-          <t>Ubuntu's 'auto' hides Windows for good after one rebuild without it. A stale Windows entry reads PROBLEM; the verify then undoes the fix. grub.cfg at 0600 (GRUB password): ERROR for a user. A cold start straight after a VBox restore skipped the menu on this host: demo with a warm reboot. On 2026-10-25 a warm reboot showed the menu for only about 3 s (the countdown ran fast): press an arrow key to hold it.</t>
+          <t>Ubuntu's 'auto' hides Windows for good after one rebuild without it. A stale Windows entry reads PROBLEM; the verify then undoes the fix. grub.cfg at 0600 (GRUB password): ERROR for a user. A cold start straight after a VBox restore skipped the menu on this host: demo with a warm reboot. On 2026-10-25 a warm reboot showed the menu for only about 0.6 s (the host's clock): tap Up from the VirtualBox logo on to hold it.</t>
         </is>
       </c>
       <c r="O19" s="12" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
-          <t>A real dual-boot machine; another release. The demo on 2026-11-03 starts from VBox snapshot grub-trap.</t>
+          <t>A real dual-boot machine; another release. The live demo on 2026-11-03 starts from VBox snapshot demo-start.</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -6802,23 +6802,60 @@
         </is>
       </c>
     </row>
-    <row r="86"/>
-    <row r="87" ht="270" customHeight="1">
-      <c r="A87" s="22" t="inlineStr">
-        <is>
-          <t>Times are IST (UTC+05:30). The logs themselves record UTC. Rows from 2026-09-07 23:35 to 2026-09-10 are records in evidence/ubuntu-26.04-2026-09-10.jsonl, copied off the VM on 2026-10-03; rows from 2026-10-04 are in evidence/ubuntu-26.04-2026-10-04.jsonl, rows from 2026-10-06 in evidence/ubuntu-26.04-2026-10-06.jsonl, and rows from 2026-10-07 in evidence/ubuntu-22.10-2026-10-07.jsonl and, from 12:13, evidence/ubuntu-22.10-2026-10-07-2.jsonl (the 22.10 VM, KineticServer). Rows from 2026-10-08 19:56 are the procedure runs, in evidence/ubuntu-22.10-2026-10-09.jsonl, copied from the service's own log, /var/log/sf3000/runs.jsonl. Rows from 2026-10-10 15:15 and 15:16 are lines 10 to 12 of evidence/ubuntu-22.10-2026-10-10.jsonl, whose first nine lines are the 2026-10-09 file again. Rows from 2026-10-10 16:33 are visit 1 of the upgrade, in evidence/ubuntu-22.10-2026-10-10-2.jsonl. The row from 18:40 is visit 2, line 3 of evidence/ubuntu-22.10-2026-10-10-3.jsonl, whose first two lines are visit 1's file again. The row from 20:00 is visit 3, line 4 of evidence/ubuntu-22.10-2026-10-10-4.jsonl, whose first three lines are visit 2's file again. The rows from 23:26 and 23:42 are Runs E and F, lines 5 and 6 of evidence/ubuntu-22.10-2026-10-10-5.jsonl, whose first four lines are visit 3's file again. The row from 2026-10-11 01:13 is Run G, line 7 of evidence/ubuntu-22.10-2026-10-11.jsonl, whose first six lines are the 2026-10-10 -5 file again. The rows from 2026-10-14 17:09 and 17:13 are visit 4, lines 8 and 9 of evidence/ubuntu-22.10-2026-10-14.jsonl, whose first seven lines are the 2026-10-11 file again. The rows from 2026-10-14 19:09 and 19:12 are Run H, lines 10 and 11 of evidence/ubuntu-22.10-2026-10-14-2.jsonl, whose first nine lines are the 2026-10-14 file again. Rows whose Evidence says 'Terminal output' have no record: the engine refuses before it logs anything, or the row is a sweep, which never logs. The six rows before 2026-09-07 23:35 come from commit messages: the VM's log was reset on the evening of 2026-09-07, before anyone copied it. Add one row per run from now on, pointing at its evidence file and line. The rows from 2026-10-16 17:10 to 17:17 are Run 1 of tests/efi-proof on KineticDesktop, an EFI 22.10 desktop VM, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16.jsonl. The rows from 18:03 to 18:10 are Run 2, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-2.jsonl: a file of its own, because the VM went back to its efi-ready snapshot between the runs. The rows from 2026-10-16 19:29 to 19:46 are tests/grub-windows-proof on KineticDesktop, one record each in evidence/ubuntu-22.10-2026-10-16-3.jsonl to -8.jsonl: each run began from a snapshot restore, which deletes the clone's run log. The rows from 2026-10-16 20:02 to 20:08 are Run 3 of tests/efi-proof, with 03's NVIDIA packages, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-9.jsonl. The rows from 2026-10-16 22:07 to 22:15 are the lab kit's test and --cancel after a real cut-off, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-10.jsonl. The rows from 2026-10-14 14:07 to 2026-10-21 13:52 are lab computer MITB-IT-406-03, a real lab machine: lines 1 to 4 of evidence/lab-MITB-IT-406-03-ubuntu-22.10-2026-10-21.jsonl (its /var/log/sf3000/runs.jsonl) and line 1 of evidence/lab-MITB-IT-406-03-ubuntu-22.10-2026-10-14.jsonl (its clone's logs/runs.jsonl). Its clock is 5 h 28 min fast; their times are corrected to the real time. The rows from 2026-10-25 14:59 are Runs 7 and 8 of tests/grub-windows-proof, the box with a summary (branch confirm-summary, a298fc9), lines 1 and 2 of evidence/ubuntu-22.10-2026-10-25.jsonl.</t>
-        </is>
-      </c>
-      <c r="B87" s="23" t="n"/>
-      <c r="C87" s="23" t="n"/>
-      <c r="D87" s="23" t="n"/>
-      <c r="E87" s="23" t="n"/>
-      <c r="F87" s="23" t="n"/>
-      <c r="G87" s="24" t="n"/>
+    <row r="86" ht="70" customHeight="1">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-25 15:24</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>c4d67cc</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>windows-missing-from-grub</t>
+        </is>
+      </c>
+      <c r="E86" s="10" t="inlineStr">
+        <is>
+          <t>healed</t>
+        </is>
+      </c>
+      <c r="F86" s="10" t="inlineStr">
+        <is>
+          <t>A timed rehearsal of the live demo from VBox snapshot demo-start (grub-trap with the clone at c4d67cc), scripted over SSH. Reboot with the fault 50 s (no menu); sweep 3 s; --fix to healed 14 s; reboot after 44 s; check-windows 47 s, no difference. GRUB's menu is up only about 0.6 s on this host; tapping Up from the VirtualBox logo on held it.</t>
+        </is>
+      </c>
+      <c r="G86" s="10" t="inlineStr">
+        <is>
+          <t>evidence/ubuntu-22.10-2026-10-25-2.jsonl, line 1; timeline and screenshots in logs/demo-rehearsal-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87"/>
+    <row r="88" ht="270" customHeight="1">
+      <c r="A88" s="22" t="inlineStr">
+        <is>
+          <t>Times are IST (UTC+05:30). The logs themselves record UTC. Rows from 2026-09-07 23:35 to 2026-09-10 are records in evidence/ubuntu-26.04-2026-09-10.jsonl, copied off the VM on 2026-10-03; rows from 2026-10-04 are in evidence/ubuntu-26.04-2026-10-04.jsonl, rows from 2026-10-06 in evidence/ubuntu-26.04-2026-10-06.jsonl, and rows from 2026-10-07 in evidence/ubuntu-22.10-2026-10-07.jsonl and, from 12:13, evidence/ubuntu-22.10-2026-10-07-2.jsonl (the 22.10 VM, KineticServer). Rows from 2026-10-08 19:56 are the procedure runs, in evidence/ubuntu-22.10-2026-10-09.jsonl, copied from the service's own log, /var/log/sf3000/runs.jsonl. Rows from 2026-10-10 15:15 and 15:16 are lines 10 to 12 of evidence/ubuntu-22.10-2026-10-10.jsonl, whose first nine lines are the 2026-10-09 file again. Rows from 2026-10-10 16:33 are visit 1 of the upgrade, in evidence/ubuntu-22.10-2026-10-10-2.jsonl. The row from 18:40 is visit 2, line 3 of evidence/ubuntu-22.10-2026-10-10-3.jsonl, whose first two lines are visit 1's file again. The row from 20:00 is visit 3, line 4 of evidence/ubuntu-22.10-2026-10-10-4.jsonl, whose first three lines are visit 2's file again. The rows from 23:26 and 23:42 are Runs E and F, lines 5 and 6 of evidence/ubuntu-22.10-2026-10-10-5.jsonl, whose first four lines are visit 3's file again. The row from 2026-10-11 01:13 is Run G, line 7 of evidence/ubuntu-22.10-2026-10-11.jsonl, whose first six lines are the 2026-10-10 -5 file again. The rows from 2026-10-14 17:09 and 17:13 are visit 4, lines 8 and 9 of evidence/ubuntu-22.10-2026-10-14.jsonl, whose first seven lines are the 2026-10-11 file again. The rows from 2026-10-14 19:09 and 19:12 are Run H, lines 10 and 11 of evidence/ubuntu-22.10-2026-10-14-2.jsonl, whose first nine lines are the 2026-10-14 file again. Rows whose Evidence says 'Terminal output' have no record: the engine refuses before it logs anything, or the row is a sweep, which never logs. The six rows before 2026-09-07 23:35 come from commit messages: the VM's log was reset on the evening of 2026-09-07, before anyone copied it. Add one row per run from now on, pointing at its evidence file and line. The rows from 2026-10-16 17:10 to 17:17 are Run 1 of tests/efi-proof on KineticDesktop, an EFI 22.10 desktop VM, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16.jsonl. The rows from 18:03 to 18:10 are Run 2, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-2.jsonl: a file of its own, because the VM went back to its efi-ready snapshot between the runs. The rows from 2026-10-16 19:29 to 19:46 are tests/grub-windows-proof on KineticDesktop, one record each in evidence/ubuntu-22.10-2026-10-16-3.jsonl to -8.jsonl: each run began from a snapshot restore, which deletes the clone's run log. The rows from 2026-10-16 20:02 to 20:08 are Run 3 of tests/efi-proof, with 03's NVIDIA packages, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-9.jsonl. The rows from 2026-10-16 22:07 to 22:15 are the lab kit's test and --cancel after a real cut-off, lines 1 to 3 of evidence/ubuntu-22.10-2026-10-16-10.jsonl. The rows from 2026-10-14 14:07 to 2026-10-21 13:52 are lab computer MITB-IT-406-03, a real lab machine: lines 1 to 4 of evidence/lab-MITB-IT-406-03-ubuntu-22.10-2026-10-21.jsonl (its /var/log/sf3000/runs.jsonl) and line 1 of evidence/lab-MITB-IT-406-03-ubuntu-22.10-2026-10-14.jsonl (its clone's logs/runs.jsonl). Its clock is 5 h 28 min fast; their times are corrected to the real time. The rows from 2026-10-25 14:59 are Runs 7 and 8 of tests/grub-windows-proof, the box with a summary (branch confirm-summary, a298fc9), lines 1 and 2 of evidence/ubuntu-22.10-2026-10-25.jsonl. The row from 2026-10-25 15:24 is a timed demo rehearsal, line 1 of evidence/ubuntu-22.10-2026-10-25-2.jsonl.</t>
+        </is>
+      </c>
+      <c r="B88" s="23" t="n"/>
+      <c r="C88" s="23" t="n"/>
+      <c r="D88" s="23" t="n"/>
+      <c r="E88" s="23" t="n"/>
+      <c r="F88" s="23" t="n"/>
+      <c r="G88" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A87:G87"/>
+    <mergeCell ref="A88:G88"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>